<commit_message>
Adiciona base de queimadas
</commit_message>
<xml_diff>
--- a/bases_levantamento.xlsx
+++ b/bases_levantamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lucas\Documents\tcc_co2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C5B6BB6-B190-4C35-BE9C-FCC7F42EEDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E920469F-874A-46F7-AA00-4FA05A16CFF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-10395" windowWidth="16440" windowHeight="28320" xr2:uid="{33A1FE18-2648-4A64-916A-DC6446327A4C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{33A1FE18-2648-4A64-916A-DC6446327A4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="51">
   <si>
     <t>Base</t>
   </si>
@@ -51,15 +51,9 @@
     <t>frota veiculos</t>
   </si>
   <si>
-    <t>denatran</t>
-  </si>
-  <si>
     <t>ibge</t>
   </si>
   <si>
-    <t>pib per capita</t>
-  </si>
-  <si>
     <t>rebanho</t>
   </si>
   <si>
@@ -123,10 +117,67 @@
     <t>Mt CO2e -&gt; 1 = 1000Kg</t>
   </si>
   <si>
-    <t>Pipeline</t>
-  </si>
-  <si>
-    <t>OK</t>
+    <t>Facilidades</t>
+  </si>
+  <si>
+    <t>Dificuldades</t>
+  </si>
+  <si>
+    <t>Possivel Causa ?</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>Nao</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://brasil.mapbiomas.org/estatisticas/</t>
+  </si>
+  <si>
+    <t>https://plataforma.seeg.eco.br/?yearRange%5B0%5D=1990&amp;yearRange%5B1%5D=2023&amp;emissionType%5B0%5D=1&amp;gas=8&amp;groupBy=Sector&amp;rankBy=State&amp;filtersTab=highlights&amp;statisticsTab=historical</t>
+  </si>
+  <si>
+    <t>https://basedosdados.org/dataset/61d592ca-5aec-4f66-b8eb-f7b894a29b66?table=3f0d609e-c85d-4daf-845f-08dd502665b2</t>
+  </si>
+  <si>
+    <t>denatran/min. Infraestrutura</t>
+  </si>
+  <si>
+    <t>https://www.ibge.gov.br/estatisticas/economicas/agricultura-e-pecuaria/9107-producao-da-pecuaria-municipal.html?=&amp;t=series-historicas</t>
+  </si>
+  <si>
+    <t>https://dados.gov.br/dados/conjuntos-dados/vendas-de-derivados-de-petroleo-e-biocombustiveis</t>
+  </si>
+  <si>
+    <t>https://portal.inmet.gov.br/dadoshistoricos</t>
+  </si>
+  <si>
+    <t>https://sidra.ibge.gov.br/Tabela/5457</t>
+  </si>
+  <si>
+    <t>https://www.epe.gov.br/pt/publicacoes-dados-abertos/publicacoes/consumo-de-energia-eletrica</t>
+  </si>
+  <si>
+    <t>Queimadas</t>
+  </si>
+  <si>
+    <t>Terra Brasilis / INPE</t>
+  </si>
+  <si>
+    <t>FRP</t>
+  </si>
+  <si>
+    <t>https://terrabrasilis.dpi.inpe.br/queimadas/bdqueimadas/#exportar-dados</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>problemas respiratorios fiocruz</t>
   </si>
 </sst>
 </file>
@@ -137,13 +188,6 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -162,13 +206,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -180,26 +238,39 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -512,17 +583,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2C43ABD-1087-4CDD-AB50-12882E517378}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.28515625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -536,13 +612,22 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -553,16 +638,19 @@
         <v>2024</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -575,96 +663,111 @@
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="E3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="1">
         <v>2003</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>2023</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="4" t="s">
+      <c r="D4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1">
-        <v>2002</v>
+        <v>1974</v>
       </c>
       <c r="C5" s="1">
         <v>2023</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="B6" s="1">
+        <v>1990</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="1">
-        <v>1974</v>
-      </c>
-      <c r="C6" s="1">
-        <v>2023</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1">
-        <v>1990</v>
+        <v>2000</v>
       </c>
       <c r="C7" s="1">
         <v>2025</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1">
         <v>2000</v>
@@ -673,117 +776,149 @@
         <v>2025</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1988</v>
+      </c>
+      <c r="C9" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1974</v>
+      </c>
+      <c r="C10" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="1">
+        <v>2004</v>
+      </c>
+      <c r="C11" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="6">
+        <v>2003</v>
+      </c>
+      <c r="C12" s="6">
+        <v>2023</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="1">
-        <v>2000</v>
-      </c>
-      <c r="C9" s="1">
+      <c r="B18" s="5">
+        <v>2008</v>
+      </c>
+      <c r="C18" s="5">
         <v>2025</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="3">
-        <v>2008</v>
-      </c>
-      <c r="C10" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="1">
-        <v>1988</v>
-      </c>
-      <c r="C11" s="1">
-        <v>2024</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="D18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="1">
-        <v>1974</v>
-      </c>
-      <c r="C12" s="1">
-        <v>2024</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="1">
-        <v>2004</v>
-      </c>
-      <c r="C13" s="1">
-        <v>2025</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B16">
-        <f>LARGE(B2:B13,1)</f>
-        <v>2008</v>
-      </c>
-      <c r="C16">
-        <f>SMALL(C2:C13,1)</f>
-        <v>2023</v>
+      <c r="G18" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{C216983A-3A18-488E-A84B-914CB31AF6CA}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{DC74C863-ABA5-4A62-B886-56C2B2751210}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{79B7708C-B87E-47A2-82CD-6D3C22575723}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{DB4D89A3-FCBB-47E7-B797-4C7337DA5DE7}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{28DC1E20-2151-41ED-BCC5-7EC51E3BBE58}"/>
+    <hyperlink ref="F7" r:id="rId6" xr:uid="{6B2A9C91-5773-435F-A52F-945DD10EA1D5}"/>
+    <hyperlink ref="F8" r:id="rId7" xr:uid="{93CC530D-BE7B-4BA1-978D-5CCCC3DE4557}"/>
+    <hyperlink ref="F9" r:id="rId8" xr:uid="{1181BD6F-5DAC-4B46-BBB7-B7A0A17DDF1C}"/>
+    <hyperlink ref="F10" r:id="rId9" xr:uid="{F6EBB35D-7BE1-4791-98E9-D3C8CA6A5161}"/>
+    <hyperlink ref="F11" r:id="rId10" xr:uid="{9F3E5380-7AB4-41E9-9CC3-0270F9402257}"/>
+    <hyperlink ref="F12" r:id="rId11" location="exportar-dados" xr:uid="{364BB60B-B7E0-433B-89FA-D6DB6703048B}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajusta recorte para 2004, remove internacoes e adiciona heatmaps
</commit_message>
<xml_diff>
--- a/bases_levantamento.xlsx
+++ b/bases_levantamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lucas\Documents\tcc_co2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E920469F-874A-46F7-AA00-4FA05A16CFF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92101D94-14F8-4BAB-879E-79AD79DD050F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{33A1FE18-2648-4A64-916A-DC6446327A4C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="71">
   <si>
     <t>Base</t>
   </si>
@@ -69,9 +69,6 @@
     <t>MapBiomas(SEEG)</t>
   </si>
   <si>
-    <t>internacoes respiratorias</t>
-  </si>
-  <si>
     <t>datasus</t>
   </si>
   <si>
@@ -178,6 +175,69 @@
   </si>
   <si>
     <t>problemas respiratorios fiocruz</t>
+  </si>
+  <si>
+    <t>http://info.gripe.fiocruz.br/</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Site indisponivel</t>
+  </si>
+  <si>
+    <t>fiocruz / infogripe</t>
+  </si>
+  <si>
+    <t>https://datasus.saude.gov.br/acesso-a-informacao/morbidade-hospitalar-do-sus-sih-sus/</t>
+  </si>
+  <si>
+    <t>Filtros limitados, download separado por ano, dados faltantes</t>
+  </si>
+  <si>
+    <t>Secas ambientais</t>
+  </si>
+  <si>
+    <t>Agência Nacional de Águas e Saneamento Básico (ANA)</t>
+  </si>
+  <si>
+    <t>https://monitordesecas.ana.gov.br/dados-tabulares?tipo=8&amp;area=5</t>
+  </si>
+  <si>
+    <t>Dados começam a partir de 2014 somente no nordeste a partir de 2020 em outras regiões</t>
+  </si>
+  <si>
+    <t>IDH</t>
+  </si>
+  <si>
+    <t>UNDP</t>
+  </si>
+  <si>
+    <t>https://www.undp.org/pt/brazil/desenvolvimento-humano/painel-idhm</t>
+  </si>
+  <si>
+    <t>Dados intervalados (CENSO) e excesso de dados faltantes</t>
+  </si>
+  <si>
+    <t>Rendimento medio mensal</t>
+  </si>
+  <si>
+    <t>IBGE</t>
+  </si>
+  <si>
+    <t>https://www.ibge.gov.br/estatisticas/sociais/rendimento-despesa-e-consumo/9127-pesquisa-nacional-por-amostra-de-domicilios.html?=&amp;t=series-historicas</t>
+  </si>
+  <si>
+    <t>Dados somente até 2015</t>
+  </si>
+  <si>
+    <t>Morbidade hospitalar (respiratoria)</t>
+  </si>
+  <si>
+    <t>Processo de download complicado pois precisava fazer uma solicitacao, entrar numa fila e aguardar um email para cada ano baixado</t>
+  </si>
+  <si>
+    <t>Downloads de arquivos separados pra cada estacao meteorológica (+ 10 mil arquivos)</t>
   </si>
 </sst>
 </file>
@@ -253,20 +313,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -583,19 +643,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2C43ABD-1087-4CDD-AB50-12882E517378}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.28515625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="41.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -612,19 +672,19 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -640,14 +700,14 @@
       <c r="D2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>36</v>
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -663,14 +723,14 @@
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>37</v>
+      <c r="E3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -684,16 +744,16 @@
         <v>2023</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>33</v>
+      <c r="E4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -709,14 +769,14 @@
       <c r="D5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>33</v>
+      <c r="E5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -732,19 +792,19 @@
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1">
         <v>2000</v>
@@ -755,19 +815,22 @@
       <c r="D7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>34</v>
+      <c r="E7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1">
         <v>2000</v>
@@ -778,19 +841,20 @@
       <c r="D8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="E8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="8"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="1">
         <v>1988</v>
@@ -801,19 +865,19 @@
       <c r="D9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>33</v>
+      <c r="E9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" s="1">
         <v>1974</v>
@@ -824,19 +888,19 @@
       <c r="D10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>33</v>
+      <c r="E10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1">
         <v>2004</v>
@@ -845,67 +909,193 @@
         <v>2025</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="4">
+        <v>2003</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2023</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="6">
-        <v>2003</v>
-      </c>
-      <c r="C12" s="6">
-        <v>2023</v>
-      </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="G12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="1">
+        <v>2008</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="5">
-        <v>2008</v>
-      </c>
-      <c r="C18" s="5">
-        <v>2025</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="E18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="G19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="1">
+        <v>2014</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I7:I8"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{C216983A-3A18-488E-A84B-914CB31AF6CA}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{DC74C863-ABA5-4A62-B886-56C2B2751210}"/>
@@ -918,6 +1108,11 @@
     <hyperlink ref="F10" r:id="rId9" xr:uid="{F6EBB35D-7BE1-4791-98E9-D3C8CA6A5161}"/>
     <hyperlink ref="F11" r:id="rId10" xr:uid="{9F3E5380-7AB4-41E9-9CC3-0270F9402257}"/>
     <hyperlink ref="F12" r:id="rId11" location="exportar-dados" xr:uid="{364BB60B-B7E0-433B-89FA-D6DB6703048B}"/>
+    <hyperlink ref="F19" r:id="rId12" xr:uid="{E4648C64-608B-4D2B-94B7-D207CE26BF25}"/>
+    <hyperlink ref="F18" r:id="rId13" xr:uid="{EAFCC355-366B-4A47-A6C8-E001408ACB48}"/>
+    <hyperlink ref="F20" r:id="rId14" xr:uid="{9AF61CFF-3AD6-4E82-A0B9-606E579229CF}"/>
+    <hyperlink ref="F21" r:id="rId15" xr:uid="{2D573F49-6741-44C2-9AE6-0E078FAD276F}"/>
+    <hyperlink ref="F22" r:id="rId16" xr:uid="{A8777C61-7F13-42B6-9197-B8FBD44ACB0E}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza levantamento de facilidades e dificuldades das bases
</commit_message>
<xml_diff>
--- a/bases_levantamento.xlsx
+++ b/bases_levantamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lucas\Documents\tcc_co2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCF0959-93C1-4F3B-96F7-E7CADFFE37A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718CFEC1-4134-486C-A9F7-781BF7687DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{33A1FE18-2648-4A64-916A-DC6446327A4C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="78">
   <si>
     <t>Base</t>
   </si>
@@ -234,10 +234,31 @@
     <t>Morbidade hospitalar (respiratoria)</t>
   </si>
   <si>
-    <t>Processo de download complicado pois precisava fazer uma solicitacao, entrar numa fila e aguardar um email para cada ano baixado</t>
-  </si>
-  <si>
-    <t>Downloads de arquivos separados pra cada estacao meteorológica (+ 10 mil arquivos)</t>
+    <t>Poucos tratamentos; já próxima do formato Estado–Ano</t>
+  </si>
+  <si>
+    <t>Agregação direta</t>
+  </si>
+  <si>
+    <t>Download simplificado</t>
+  </si>
+  <si>
+    <t>Estrutura com anos e animais em múltiplos níveis; precisei reconstruir a tabela antes da análise</t>
+  </si>
+  <si>
+    <t>Agregação semi-direta</t>
+  </si>
+  <si>
+    <t>Ajuste na granularidade de tempo (base mensal)</t>
+  </si>
+  <si>
+    <t>Conversão para Estado–Ano</t>
+  </si>
+  <si>
+    <t>Processo de download com muitas etapas para cada ano. Muitos arquivos; leitura em partes;</t>
+  </si>
+  <si>
+    <t>Excesso de arquivos, colunas inconsistentes, diversas agregações pois um unico estado possui mais de uma estação; leitura em partes</t>
   </si>
 </sst>
 </file>
@@ -296,7 +317,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -318,6 +339,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -644,8 +671,8 @@
     <col min="5" max="5" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="41.28515625" style="1" customWidth="1"/>
     <col min="7" max="7" width="20.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18.140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="41.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="43.42578125" style="6" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -700,8 +727,14 @@
       <c r="G2" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -722,6 +755,12 @@
       </c>
       <c r="G3" s="1" t="s">
         <v>48</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -746,8 +785,14 @@
       <c r="G4" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -768,6 +813,12 @@
       </c>
       <c r="G5" s="1" t="s">
         <v>32</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -792,6 +843,12 @@
       <c r="G6" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="H6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -809,14 +866,17 @@
       <c r="E7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="8" t="s">
         <v>33</v>
       </c>
+      <c r="H7" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="I7" s="7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -835,12 +895,9 @@
       <c r="E8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
       <c r="I8" s="7"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -859,11 +916,17 @@
       <c r="E9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="8" t="s">
         <v>32</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -882,14 +945,12 @@
       <c r="E10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F10" s="9"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>25</v>
       </c>
@@ -911,8 +972,14 @@
       <c r="G11" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="H11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>44</v>
       </c>
@@ -934,8 +1001,11 @@
       <c r="G12" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="H12" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="I12" s="6" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1084,8 +1154,15 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="H7:H8"/>
     <mergeCell ref="I7:I8"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="G7:G8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{C216983A-3A18-488E-A84B-914CB31AF6CA}"/>
@@ -1094,16 +1171,14 @@
     <hyperlink ref="F5" r:id="rId4" xr:uid="{DB4D89A3-FCBB-47E7-B797-4C7337DA5DE7}"/>
     <hyperlink ref="F6" r:id="rId5" xr:uid="{28DC1E20-2151-41ED-BCC5-7EC51E3BBE58}"/>
     <hyperlink ref="F7" r:id="rId6" xr:uid="{6B2A9C91-5773-435F-A52F-945DD10EA1D5}"/>
-    <hyperlink ref="F8" r:id="rId7" xr:uid="{93CC530D-BE7B-4BA1-978D-5CCCC3DE4557}"/>
-    <hyperlink ref="F9" r:id="rId8" xr:uid="{1181BD6F-5DAC-4B46-BBB7-B7A0A17DDF1C}"/>
-    <hyperlink ref="F10" r:id="rId9" xr:uid="{F6EBB35D-7BE1-4791-98E9-D3C8CA6A5161}"/>
-    <hyperlink ref="F11" r:id="rId10" xr:uid="{9F3E5380-7AB4-41E9-9CC3-0270F9402257}"/>
-    <hyperlink ref="F12" r:id="rId11" location="exportar-dados" xr:uid="{364BB60B-B7E0-433B-89FA-D6DB6703048B}"/>
-    <hyperlink ref="F19" r:id="rId12" xr:uid="{E4648C64-608B-4D2B-94B7-D207CE26BF25}"/>
-    <hyperlink ref="F18" r:id="rId13" xr:uid="{EAFCC355-366B-4A47-A6C8-E001408ACB48}"/>
-    <hyperlink ref="F20" r:id="rId14" xr:uid="{9AF61CFF-3AD6-4E82-A0B9-606E579229CF}"/>
-    <hyperlink ref="F21" r:id="rId15" xr:uid="{2D573F49-6741-44C2-9AE6-0E078FAD276F}"/>
-    <hyperlink ref="F22" r:id="rId16" xr:uid="{A8777C61-7F13-42B6-9197-B8FBD44ACB0E}"/>
+    <hyperlink ref="F9" r:id="rId7" xr:uid="{F6EBB35D-7BE1-4791-98E9-D3C8CA6A5161}"/>
+    <hyperlink ref="F11" r:id="rId8" xr:uid="{9F3E5380-7AB4-41E9-9CC3-0270F9402257}"/>
+    <hyperlink ref="F12" r:id="rId9" location="exportar-dados" xr:uid="{364BB60B-B7E0-433B-89FA-D6DB6703048B}"/>
+    <hyperlink ref="F19" r:id="rId10" xr:uid="{E4648C64-608B-4D2B-94B7-D207CE26BF25}"/>
+    <hyperlink ref="F18" r:id="rId11" xr:uid="{EAFCC355-366B-4A47-A6C8-E001408ACB48}"/>
+    <hyperlink ref="F20" r:id="rId12" xr:uid="{9AF61CFF-3AD6-4E82-A0B9-606E579229CF}"/>
+    <hyperlink ref="F21" r:id="rId13" xr:uid="{2D573F49-6741-44C2-9AE6-0E078FAD276F}"/>
+    <hyperlink ref="F22" r:id="rId14" xr:uid="{A8777C61-7F13-42B6-9197-B8FBD44ACB0E}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>